<commit_message>
updated requirenements of python
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>45745.4330791618</v>
+        <v>45745.43307916667</v>
       </c>
     </row>
     <row r="3">
@@ -502,6 +502,25 @@
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Anshuman Prajapati</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>anshumandoc16@gmail.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2c4d5989afa2b4793ee305ab9caec4431e8ef9567fdcfd334bf29322b0ba7a59</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>